<commit_message>
Add step-by-step solution notes to Project Investment Example 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016LewYKKY4R5TZnd6fZ2qK4
</commit_message>
<xml_diff>
--- a/DCF_Project_Investment_Completed.xlsx
+++ b/DCF_Project_Investment_Completed.xlsx
@@ -8955,7 +8955,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:Q34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" style="261" bestFit="1" customWidth="1"/>
@@ -9765,8 +9765,89 @@
         <v>104351.53626634751</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="D31" s="285"/>
+    <row r="23" spans="1:13">
+      <c r="A23" s="279" t="inlineStr">
+        <is>
+          <t>HOW THIS PAGE WAS SOLVED (step by step)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
+      <c r="A24" s="261" t="inlineStr">
+        <is>
+          <t>Step 1 - Incremental profit per week (row 9): Profit Rate x Incremental Sales/Wk.  e.g. E9 = $B$8*E7 = 25% x 4,000 = $1,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
+      <c r="A25" s="261" t="inlineStr">
+        <is>
+          <t>Step 2 - Year 0 (column B): the capital spent, entered as a negative.  B19 = -E10 = (800,000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
+      <c r="A26" s="261" t="inlineStr">
+        <is>
+          <t>Step 3 - Year 1 (column C): weekly profit x 52 weeks.  C19 = E9*$B$14 = 1,000 x 52 = 52,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
+      <c r="A27" s="261" t="inlineStr">
+        <is>
+          <t>Step 4 - Years 2 to 10 (D:L): grow the prior year by the 1.5% growth assumption.  D19 = C19*(1+$B$10) = 52,780 ... drag right to L</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
+      <c r="A28" s="261" t="inlineStr">
+        <is>
+          <t>Step 5 - Sum of Years (column M): add Years 1-10 only (not Year 0).  M19 = SUM(C19:L19) = 556,542</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
+      <c r="A29" s="261" t="inlineStr">
+        <is>
+          <t>Step 6 - Repeat Steps 2-5 for rows 20 and 21, pointing at columns F and G above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
+      <c r="A30" s="261" t="inlineStr">
+        <is>
+          <t>Step 7 - ROC (row 11): (Sum of Cash Flows - Capital) / Capital.  E11 = (M19-E10)/E10 = -30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
+      <c r="A31" s="261" t="inlineStr">
+        <is>
+          <t>Step 8 - IRR (row 12): IRR of the full stream INCLUDING Year 0.  E12 = IRR(B19:L19) = -6.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
+      <c r="A32" s="261" t="inlineStr">
+        <is>
+          <t>Step 9 - NPV (row 13): discount Years 1-10 at 4%, then add the undiscounted Year 0 cost.  E13 = NPV($B$12,C19:L19)+B19 = (350,761)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" spans="1:13">
+      <c r="A33" s="261" t="inlineStr">
+        <is>
+          <t>Step 10 - Decide: accept projects with NPV &gt; 0 and IRR &gt; the 4% discount rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:13">
+      <c r="A34" s="279" t="inlineStr">
+        <is>
+          <t>RESULT: Only Improved Operations Management passes (NPV $49,232, IRR 26.2%, ROC 198%). Shirt Enhancement and Marketing Campaign Upgrade both lose value.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>